<commit_message>
Add per-sheet ability indices to generated Excel reference
</commit_message>
<xml_diff>
--- a/CLASS_ABILITIES.xlsx
+++ b/CLASS_ABILITIES.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archer" sheetId="1" r:id="R9212a9b4cb6b46e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleric" sheetId="2" r:id="Rb0cd6058e062413f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warrior" sheetId="3" r:id="R1dc8fc8b539d4817"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wizard" sheetId="4" r:id="Rf0a09fbf750a4534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archer" sheetId="1" r:id="R57d264d87e174cb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleric" sheetId="2" r:id="Reac5d977d17c4c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warrior" sheetId="3" r:id="R41573a6b5f8a4530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wizard" sheetId="4" r:id="Rc5de371bc3284c27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,29 +131,29 @@
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -163,52 +163,56 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ClassAbilities1" displayName="ClassAbilities1" ref="A5:D10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:D10"/>
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="Class"/>
-    <x:tableColumn id="2" name="Unlock Level"/>
-    <x:tableColumn id="3" name="Ability"/>
-    <x:tableColumn id="4" name="Description"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ClassAbilities1" displayName="ClassAbilities1" ref="A5:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E10"/>
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Index"/>
+    <x:tableColumn id="2" name="Class"/>
+    <x:tableColumn id="3" name="Unlock Level"/>
+    <x:tableColumn id="4" name="Ability"/>
+    <x:tableColumn id="5" name="Description"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClassAbilities2" displayName="ClassAbilities2" ref="A5:D12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:D12"/>
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="Class"/>
-    <x:tableColumn id="2" name="Unlock Level"/>
-    <x:tableColumn id="3" name="Ability"/>
-    <x:tableColumn id="4" name="Description"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClassAbilities2" displayName="ClassAbilities2" ref="A5:E12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E12"/>
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Index"/>
+    <x:tableColumn id="2" name="Class"/>
+    <x:tableColumn id="3" name="Unlock Level"/>
+    <x:tableColumn id="4" name="Ability"/>
+    <x:tableColumn id="5" name="Description"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ClassAbilities3" displayName="ClassAbilities3" ref="A5:D14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:D14"/>
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="Class"/>
-    <x:tableColumn id="2" name="Unlock Level"/>
-    <x:tableColumn id="3" name="Ability"/>
-    <x:tableColumn id="4" name="Description"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ClassAbilities3" displayName="ClassAbilities3" ref="A5:E14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E14"/>
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Index"/>
+    <x:tableColumn id="2" name="Class"/>
+    <x:tableColumn id="3" name="Unlock Level"/>
+    <x:tableColumn id="4" name="Ability"/>
+    <x:tableColumn id="5" name="Description"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClassAbilities4" displayName="ClassAbilities4" ref="A5:D12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:D12"/>
-  <x:tableColumns count="4">
-    <x:tableColumn id="1" name="Class"/>
-    <x:tableColumn id="2" name="Unlock Level"/>
-    <x:tableColumn id="3" name="Ability"/>
-    <x:tableColumn id="4" name="Description"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClassAbilities4" displayName="ClassAbilities4" ref="A5:E12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E12"/>
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Index"/>
+    <x:tableColumn id="2" name="Class"/>
+    <x:tableColumn id="3" name="Unlock Level"/>
+    <x:tableColumn id="4" name="Ability"/>
+    <x:tableColumn id="5" name="Description"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -412,10 +416,11 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22.75" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="90" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="90" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -423,6 +428,7 @@
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
       <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
@@ -431,19 +437,23 @@
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="8" t="str">
+        <x:v>Per sheet</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
         <x:v>Generated reference</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="str">
+      <x:c r="C3" s="8" t="str">
         <x:v>Class levels</x:v>
       </x:c>
-      <x:c r="C3" s="8" t="str">
+      <x:c r="D3" s="8" t="str">
         <x:v>All classes = basic attacks</x:v>
       </x:c>
-      <x:c r="D3" s="8" t="str">
-        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Blank level = no class-level requirement.</x:v>
+      <x:c r="E3" s="8" t="str">
+        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Indices show reference order, not permanent IDs. Blank unlock level = no class-level requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="8" customHeight="1">
@@ -451,94 +461,113 @@
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="11" t="str">
+        <x:v>Index</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
         <x:v>Class</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>Unlock Level</x:v>
       </x:c>
-      <x:c r="C5" s="11" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>Ability</x:v>
       </x:c>
-      <x:c r="D5" s="11" t="str">
+      <x:c r="E5" s="11" t="str">
         <x:v>Description</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="57" customHeight="1">
-      <x:c r="A6" s="18" t="str">
+      <x:c r="A6" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B6" s="19"/>
-      <x:c r="C6" s="18" t="str">
+      <x:c r="C6" s="18"/>
+      <x:c r="D6" s="19" t="str">
         <x:v>Strike</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str">
+      <x:c r="E6" s="19" t="str">
         <x:v>Melee ability. Melee. Range 1.41. Physical damage (weapon damage + Strength x100%). Affects: enemies. Can aim at a cell. Melee weapon or unarmed friendly. Compatible weapon range bonuses extend normal attacks.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="22" t="str">
+      <x:c r="A7" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B7" s="23"/>
-      <x:c r="C7" s="22" t="str">
+      <x:c r="C7" s="22"/>
+      <x:c r="D7" s="23" t="str">
         <x:v>Shoot</x:v>
       </x:c>
-      <x:c r="D7" s="22" t="str">
+      <x:c r="E7" s="23" t="str">
         <x:v>Ranged ability. Projectile. Range 5.00. Physical damage (weapon damage + Dexterity x60%). Affects: enemies. Can aim at a cell. Ranged weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="18" t="str">
+      <x:c r="A8" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
         <x:v>Archer</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="n">
+      <x:c r="C8" s="18" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C8" s="18" t="str">
+      <x:c r="D8" s="19" t="str">
         <x:v>Focus</x:v>
       </x:c>
-      <x:c r="D8" s="18" t="str">
+      <x:c r="E8" s="19" t="str">
         <x:v>Magic ability. Cast. Range 0.00. Focus for 2 turns. +2 Strength, +2 Dexterity, +2 Intelligence. Positive status. Affects: self. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="57" customHeight="1">
-      <x:c r="A9" s="22" t="str">
+      <x:c r="A9" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
         <x:v>Archer</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="n">
+      <x:c r="C9" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="str">
+      <x:c r="D9" s="23" t="str">
         <x:v>Multiple Arrows</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="str">
+      <x:c r="E9" s="23" t="str">
         <x:v>Ranged ability. Projectile. Range 5.00. Physical damage (3 hits × (weapon damage + Dexterity x60%)). Choose 3 targets in order; repeats allowed; confirm to fire. Affects: enemies. Ranged weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="18" t="str">
+      <x:c r="A10" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
         <x:v>Archer</x:v>
       </x:c>
-      <x:c r="B10" s="19" t="n">
+      <x:c r="C10" s="18" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C10" s="18" t="str">
+      <x:c r="D10" s="19" t="str">
         <x:v>Dagger Throw</x:v>
       </x:c>
-      <x:c r="D10" s="18" t="str">
+      <x:c r="E10" s="19" t="str">
         <x:v>Ranged ability. Projectile. Range 5.00. Physical damage (Dexterity x100%). Affects: enemies. No weapon required.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24d0cb4b5d364e72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c057f72496e474d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -550,10 +579,11 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22.75" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="90" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="90" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -561,6 +591,7 @@
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
       <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
@@ -569,19 +600,23 @@
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="8" t="str">
+        <x:v>Per sheet</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
         <x:v>Generated reference</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="str">
+      <x:c r="C3" s="8" t="str">
         <x:v>Class levels</x:v>
       </x:c>
-      <x:c r="C3" s="8" t="str">
+      <x:c r="D3" s="8" t="str">
         <x:v>All classes = basic attacks</x:v>
       </x:c>
-      <x:c r="D3" s="8" t="str">
-        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Blank level = no class-level requirement.</x:v>
+      <x:c r="E3" s="8" t="str">
+        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Indices show reference order, not permanent IDs. Blank unlock level = no class-level requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="8" customHeight="1">
@@ -589,122 +624,147 @@
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="11" t="str">
+        <x:v>Index</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
         <x:v>Class</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>Unlock Level</x:v>
       </x:c>
-      <x:c r="C5" s="11" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>Ability</x:v>
       </x:c>
-      <x:c r="D5" s="11" t="str">
+      <x:c r="E5" s="11" t="str">
         <x:v>Description</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="57" customHeight="1">
-      <x:c r="A6" s="18" t="str">
+      <x:c r="A6" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B6" s="19"/>
-      <x:c r="C6" s="18" t="str">
+      <x:c r="C6" s="18"/>
+      <x:c r="D6" s="19" t="str">
         <x:v>Strike</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str">
+      <x:c r="E6" s="19" t="str">
         <x:v>Melee ability. Melee. Range 1.41. Physical damage (weapon damage + Strength x100%). Affects: enemies. Can aim at a cell. Melee weapon or unarmed friendly. Compatible weapon range bonuses extend normal attacks.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="22" t="str">
+      <x:c r="A7" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B7" s="23"/>
-      <x:c r="C7" s="22" t="str">
+      <x:c r="C7" s="22"/>
+      <x:c r="D7" s="23" t="str">
         <x:v>Shoot</x:v>
       </x:c>
-      <x:c r="D7" s="22" t="str">
+      <x:c r="E7" s="23" t="str">
         <x:v>Ranged ability. Projectile. Range 5.00. Physical damage (weapon damage + Dexterity x60%). Affects: enemies. Can aim at a cell. Ranged weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="18" t="str">
+      <x:c r="A8" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
         <x:v>Cleric</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="n">
+      <x:c r="C8" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="18" t="str">
+      <x:c r="D8" s="19" t="str">
         <x:v>Heal</x:v>
       </x:c>
-      <x:c r="D8" s="18" t="str">
+      <x:c r="E8" s="19" t="str">
         <x:v>Magic ability. Cast. Range 5.00. Healing (25 base + Intelligence x100%). Affects: allies, self. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="22" t="str">
+      <x:c r="A9" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
         <x:v>Cleric</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="n">
+      <x:c r="C9" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="str">
+      <x:c r="D9" s="23" t="str">
         <x:v>Beam</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="str">
+      <x:c r="E9" s="23" t="str">
         <x:v>Magic ability. Cast. Range 3.00. Magical damage (10 innate + Intelligence x100%). Affects: enemies. Can aim at a cell. Line from caster toward target. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="18" t="str">
+      <x:c r="A10" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
         <x:v>Cleric</x:v>
       </x:c>
-      <x:c r="B10" s="19" t="n">
+      <x:c r="C10" s="18" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C10" s="18" t="str">
+      <x:c r="D10" s="19" t="str">
         <x:v>Focus</x:v>
       </x:c>
-      <x:c r="D10" s="18" t="str">
+      <x:c r="E10" s="19" t="str">
         <x:v>Magic ability. Cast. Range 0.00. Focus for 2 turns. +2 Strength, +2 Dexterity, +2 Intelligence. Positive status. Affects: self. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="57" customHeight="1">
-      <x:c r="A11" s="22" t="str">
+      <x:c r="A11" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
         <x:v>Cleric</x:v>
       </x:c>
-      <x:c r="B11" s="23" t="n">
+      <x:c r="C11" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C11" s="22" t="str">
+      <x:c r="D11" s="23" t="str">
         <x:v>Empower</x:v>
       </x:c>
-      <x:c r="D11" s="22" t="str">
+      <x:c r="E11" s="23" t="str">
         <x:v>Magic ability. Cast. Range 5.00. Empowered for 3 turns. +1 Strength, +1 Dexterity, +1 Intelligence, +1 Constitution, +1 Speed, +1 Movement Range. Positive status. Affects: allies, self. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="18" t="str">
+      <x:c r="A12" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
         <x:v>Cleric</x:v>
       </x:c>
-      <x:c r="B12" s="19" t="n">
+      <x:c r="C12" s="18" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C12" s="18" t="str">
+      <x:c r="D12" s="19" t="str">
         <x:v>Cleanse</x:v>
       </x:c>
-      <x:c r="D12" s="18" t="str">
+      <x:c r="E12" s="19" t="str">
         <x:v>Magic ability. Cast. Range 5.00. Remove all negative statuses; preserve positive statuses. Affects: allies, self. No weapon required.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94a9d16a45a142ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3ca1f25c2554bd8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -716,10 +776,11 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22.75" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="90" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="90" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -727,6 +788,7 @@
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
       <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
@@ -735,19 +797,23 @@
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="8" t="str">
+        <x:v>Per sheet</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
         <x:v>Generated reference</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="str">
+      <x:c r="C3" s="8" t="str">
         <x:v>Class levels</x:v>
       </x:c>
-      <x:c r="C3" s="8" t="str">
+      <x:c r="D3" s="8" t="str">
         <x:v>All classes = basic attacks</x:v>
       </x:c>
-      <x:c r="D3" s="8" t="str">
-        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Blank level = no class-level requirement.</x:v>
+      <x:c r="E3" s="8" t="str">
+        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Indices show reference order, not permanent IDs. Blank unlock level = no class-level requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="8" customHeight="1">
@@ -755,150 +821,181 @@
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="11" t="str">
+        <x:v>Index</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
         <x:v>Class</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>Unlock Level</x:v>
       </x:c>
-      <x:c r="C5" s="11" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>Ability</x:v>
       </x:c>
-      <x:c r="D5" s="11" t="str">
+      <x:c r="E5" s="11" t="str">
         <x:v>Description</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="57" customHeight="1">
-      <x:c r="A6" s="18" t="str">
+      <x:c r="A6" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B6" s="19"/>
-      <x:c r="C6" s="18" t="str">
+      <x:c r="C6" s="18"/>
+      <x:c r="D6" s="19" t="str">
         <x:v>Strike</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str">
+      <x:c r="E6" s="19" t="str">
         <x:v>Melee ability. Melee. Range 1.41. Physical damage (weapon damage + Strength x100%). Affects: enemies. Can aim at a cell. Melee weapon or unarmed friendly. Compatible weapon range bonuses extend normal attacks.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="22" t="str">
+      <x:c r="A7" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B7" s="23"/>
-      <x:c r="C7" s="22" t="str">
+      <x:c r="C7" s="22"/>
+      <x:c r="D7" s="23" t="str">
         <x:v>Shoot</x:v>
       </x:c>
-      <x:c r="D7" s="22" t="str">
+      <x:c r="E7" s="23" t="str">
         <x:v>Ranged ability. Projectile. Range 5.00. Physical damage (weapon damage + Dexterity x60%). Affects: enemies. Can aim at a cell. Ranged weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="18" t="str">
+      <x:c r="A8" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
         <x:v>Warrior</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="n">
+      <x:c r="C8" s="18" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C8" s="18" t="str">
+      <x:c r="D8" s="19" t="str">
         <x:v>Charge</x:v>
       </x:c>
-      <x:c r="D8" s="18" t="str">
+      <x:c r="E8" s="19" t="str">
         <x:v>Melee ability. Melee. Range 5.00. Physical damage (weapon damage + Strength x100%). Charges in a clear straight line and stops adjacent. Affects: enemies. Melee weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="22" t="str">
+      <x:c r="A9" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
         <x:v>Warrior</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="n">
+      <x:c r="C9" s="22" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="str">
+      <x:c r="D9" s="23" t="str">
         <x:v>Battle Stomp</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="str">
+      <x:c r="E9" s="23" t="str">
         <x:v>Melee ability. Cast. Range 1.50. Physical damage (weapon damage + Strength x100%). Radius 1.50 around caster; click caster to confirm. Affects: enemies. Melee weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="57" customHeight="1">
-      <x:c r="A10" s="18" t="str">
+      <x:c r="A10" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
         <x:v>Warrior</x:v>
       </x:c>
-      <x:c r="B10" s="19" t="n">
+      <x:c r="C10" s="18" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C10" s="18" t="str">
+      <x:c r="D10" s="19" t="str">
         <x:v>Taunt</x:v>
       </x:c>
-      <x:c r="D10" s="18" t="str">
+      <x:c r="E10" s="19" t="str">
         <x:v>Melee ability. Cast. Range 1.50. Taunted: Attack the caster if possible; otherwise pursue them for 1 turn. Negative status. Radius 1.50 around caster; click caster to confirm. Affects: enemies. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="22" t="str">
+      <x:c r="A11" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
         <x:v>Warrior</x:v>
       </x:c>
-      <x:c r="B11" s="23" t="n">
+      <x:c r="C11" s="22" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C11" s="22" t="str">
+      <x:c r="D11" s="23" t="str">
         <x:v>Multi Attack</x:v>
       </x:c>
-      <x:c r="D11" s="22" t="str">
+      <x:c r="E11" s="23" t="str">
         <x:v>Melee ability. Melee. Range 1.41. Physical damage (2 hits × (weapon damage + Strength x50%)). 2 separate hits on the same target. Affects: enemies. Melee weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
-      <x:c r="A12" s="18" t="str">
+      <x:c r="A12" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
         <x:v>Warrior</x:v>
       </x:c>
-      <x:c r="B12" s="19" t="n">
+      <x:c r="C12" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C12" s="18" t="str">
+      <x:c r="D12" s="19" t="str">
         <x:v>Counter</x:v>
       </x:c>
-      <x:c r="D12" s="18" t="str">
+      <x:c r="E12" s="19" t="str">
         <x:v>Melee ability. Cast. Range 0.00. Counter for 1 turn. After each complete damaging attack, retaliate once with your basic attack if the attacker is in range. Retaliation costs no action or opportunity reaction. Requires being able to attack; excludes terrain, damage over time, and other counters. Expires at next turn start. Positive status. Affects: self. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="57" customHeight="1">
-      <x:c r="A13" s="22" t="str">
+      <x:c r="A13" s="22" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B13" s="23" t="str">
         <x:v>Warrior</x:v>
       </x:c>
-      <x:c r="B13" s="23" t="n">
+      <x:c r="C13" s="22" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C13" s="22" t="str">
+      <x:c r="D13" s="23" t="str">
         <x:v>Swipe</x:v>
       </x:c>
-      <x:c r="D13" s="22" t="str">
+      <x:c r="E13" s="23" t="str">
         <x:v>Melee ability. Melee. Range 1.00. Physical damage (weapon damage + Strength x100%). Click an orthogonally adjacent cell; hit a 3-cell row across that direction. Affects: enemies. Can aim at a cell. Area: line in front, 3-cell span. Melee weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
-      <x:c r="A14" s="18" t="str">
+      <x:c r="A14" s="18" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B14" s="19" t="str">
         <x:v>Warrior</x:v>
       </x:c>
-      <x:c r="B14" s="19" t="n">
+      <x:c r="C14" s="18" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C14" s="18" t="str">
+      <x:c r="D14" s="19" t="str">
         <x:v>Ram</x:v>
       </x:c>
-      <x:c r="D14" s="18" t="str">
+      <x:c r="E14" s="19" t="str">
         <x:v>Melee ability. Melee. Range 1.00. Physical damage (Strength x100%), Push up to 2 tiles away; walls and board edges deal 1 collision damage; hitting a unit stops the push and deals 1 to both (armor applies). No chain push, terrain entry effects, or opportunity attacks. Affects: enemies. No weapon required.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c59d42d75434b45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c00eeaddc924b30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -910,10 +1007,11 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22.75" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="90" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="90" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -921,6 +1019,7 @@
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
       <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="5" t="str">
@@ -929,19 +1028,23 @@
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
+      <x:c r="E2" s="6"/>
     </x:row>
     <x:row r="3" ht="42" customHeight="1">
       <x:c r="A3" s="8" t="str">
+        <x:v>Per sheet</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
         <x:v>Generated reference</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="str">
+      <x:c r="C3" s="8" t="str">
         <x:v>Class levels</x:v>
       </x:c>
-      <x:c r="C3" s="8" t="str">
+      <x:c r="D3" s="8" t="str">
         <x:v>All classes = basic attacks</x:v>
       </x:c>
-      <x:c r="D3" s="8" t="str">
-        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Blank level = no class-level requirement.</x:v>
+      <x:c r="E3" s="8" t="str">
+        <x:v>Edit resources in Godot. Saved changes update this file. Close and reopen Excel to see updates. Indices show reference order, not permanent IDs. Blank unlock level = no class-level requirement.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="8" customHeight="1">
@@ -949,122 +1052,147 @@
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
       <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="11" t="str">
+        <x:v>Index</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
         <x:v>Class</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
+      <x:c r="C5" s="11" t="str">
         <x:v>Unlock Level</x:v>
       </x:c>
-      <x:c r="C5" s="11" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>Ability</x:v>
       </x:c>
-      <x:c r="D5" s="11" t="str">
+      <x:c r="E5" s="11" t="str">
         <x:v>Description</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="57" customHeight="1">
-      <x:c r="A6" s="18" t="str">
+      <x:c r="A6" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B6" s="19" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B6" s="19"/>
-      <x:c r="C6" s="18" t="str">
+      <x:c r="C6" s="18"/>
+      <x:c r="D6" s="19" t="str">
         <x:v>Strike</x:v>
       </x:c>
-      <x:c r="D6" s="18" t="str">
+      <x:c r="E6" s="19" t="str">
         <x:v>Melee ability. Melee. Range 1.41. Physical damage (weapon damage + Strength x100%). Affects: enemies. Can aim at a cell. Melee weapon or unarmed friendly. Compatible weapon range bonuses extend normal attacks.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="22" t="str">
+      <x:c r="A7" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B7" s="23" t="str">
         <x:v>All classes</x:v>
       </x:c>
-      <x:c r="B7" s="23"/>
-      <x:c r="C7" s="22" t="str">
+      <x:c r="C7" s="22"/>
+      <x:c r="D7" s="23" t="str">
         <x:v>Shoot</x:v>
       </x:c>
-      <x:c r="D7" s="22" t="str">
+      <x:c r="E7" s="23" t="str">
         <x:v>Ranged ability. Projectile. Range 5.00. Physical damage (weapon damage + Dexterity x60%). Affects: enemies. Can aim at a cell. Ranged weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="18" t="str">
+      <x:c r="A8" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="19" t="str">
         <x:v>Wizard</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="n">
+      <x:c r="C8" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="18" t="str">
+      <x:c r="D8" s="19" t="str">
         <x:v>Ice Shard</x:v>
       </x:c>
-      <x:c r="D8" s="18" t="str">
+      <x:c r="E8" s="19" t="str">
         <x:v>Magic ability. Projectile. Range 5.00. Magical damage (15 innate + Intelligence x100%), Slow: Reduce Movement Range by 30% for 2 turns. Negative status. Affects: enemies. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="57" customHeight="1">
-      <x:c r="A9" s="22" t="str">
+      <x:c r="A9" s="22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B9" s="23" t="str">
         <x:v>Wizard</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="n">
+      <x:c r="C9" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C9" s="22" t="str">
+      <x:c r="D9" s="23" t="str">
         <x:v>Searing Dagger</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="str">
+      <x:c r="E9" s="23" t="str">
         <x:v>Magic ability. Projectile. Range 8.00. Magical damage (15 innate + Intelligence x100%), Burning: 1 magical damage at turn start for 2 turns. Negative status. Affects: enemies. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="18" t="str">
+      <x:c r="A10" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B10" s="19" t="str">
         <x:v>Wizard</x:v>
       </x:c>
-      <x:c r="B10" s="19" t="n">
+      <x:c r="C10" s="18" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C10" s="18" t="str">
+      <x:c r="D10" s="19" t="str">
         <x:v>Slow</x:v>
       </x:c>
-      <x:c r="D10" s="18" t="str">
+      <x:c r="E10" s="19" t="str">
         <x:v>Magic ability. Cast. Range 5.00. Slow: Reduce Movement Range by 30% for 2 turns. Negative status. Affects: enemies. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="22" t="str">
+      <x:c r="A11" s="22" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B11" s="23" t="str">
         <x:v>Wizard</x:v>
       </x:c>
-      <x:c r="B11" s="23" t="n">
+      <x:c r="C11" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C11" s="22" t="str">
+      <x:c r="D11" s="23" t="str">
         <x:v>Fireball</x:v>
       </x:c>
-      <x:c r="D11" s="22" t="str">
+      <x:c r="E11" s="23" t="str">
         <x:v>Magic ability. Projectile. Range 8.00. Magical damage (20 innate + Intelligence x100%). Affects: enemies. Can aim at a cell. Area: circle, 7-cell span. No weapon required.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
-      <x:c r="A12" s="18" t="str">
+      <x:c r="A12" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
         <x:v>Wizard</x:v>
       </x:c>
-      <x:c r="B12" s="19" t="n">
+      <x:c r="C12" s="18" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C12" s="18" t="str">
+      <x:c r="D12" s="19" t="str">
         <x:v>Beam</x:v>
       </x:c>
-      <x:c r="D12" s="18" t="str">
+      <x:c r="E12" s="19" t="str">
         <x:v>Magic ability. Cast. Range 3.00. Magical damage (10 innate + Intelligence x100%). Affects: enemies. Can aim at a cell. Line from caster toward target. No weapon required.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A2:E2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a4dbe2d26df4e5e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R092dd6e20e594019"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Bloodlust warrior ability with reusable on-kill status rewards
</commit_message>
<xml_diff>
--- a/CLASS_ABILITIES.xlsx
+++ b/CLASS_ABILITIES.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archer" sheetId="1" r:id="R57d264d87e174cb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleric" sheetId="2" r:id="Reac5d977d17c4c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warrior" sheetId="3" r:id="R41573a6b5f8a4530"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wizard" sheetId="4" r:id="Rc5de371bc3284c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archer" sheetId="1" r:id="R5920734ec8894147"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleric" sheetId="2" r:id="R15c9d9eee8ae4ef8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warrior" sheetId="3" r:id="R9f8372037e18495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wizard" sheetId="4" r:id="R0ad989e67db14c82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -191,8 +191,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ClassAbilities3" displayName="ClassAbilities3" ref="A5:E14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:E14"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ClassAbilities3" displayName="ClassAbilities3" ref="A5:E15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:E15"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Index"/>
     <x:tableColumn id="2" name="Class"/>
@@ -567,7 +567,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c057f72496e474d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3d11dc90ee946fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -764,7 +764,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3ca1f25c2554bd8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bd255d0efe6422c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -887,7 +887,7 @@
         <x:v>Melee ability. Melee. Range 5.00. Physical damage (weapon damage + Strength x100%). Charges in a clear straight line and stops adjacent. Affects: enemies. Melee weapon required.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="42" customHeight="1">
+    <x:row r="9" ht="57" customHeight="1">
       <x:c r="A9" s="22" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -895,16 +895,16 @@
         <x:v>Warrior</x:v>
       </x:c>
       <x:c r="C9" s="22" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
-        <x:v>Battle Stomp</x:v>
+        <x:v>Bloodlust</x:v>
       </x:c>
       <x:c r="E9" s="23" t="str">
-        <x:v>Melee ability. Cast. Range 1.50. Physical damage (weapon damage + Strength x100%). Radius 1.50 around caster; click caster to confirm. Affects: enemies. Melee weapon required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="57" customHeight="1">
+        <x:v>Melee ability. Melee. Range 1.41. Physical damage (weapon damage + Strength x100%), On kill: caster gains Strength Up ×2 (Strength Up: +1 Strength per stack. Until battle ends. Positive status). Affects: enemies. Melee weapon required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="18" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -912,16 +912,16 @@
         <x:v>Warrior</x:v>
       </x:c>
       <x:c r="C10" s="18" t="n">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D10" s="19" t="str">
-        <x:v>Taunt</x:v>
+        <x:v>Battle Stomp</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>Melee ability. Cast. Range 1.50. Taunted: Attack the caster if possible; otherwise pursue them for 1 turn. Negative status. Radius 1.50 around caster; click caster to confirm. Affects: enemies. No weapon required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="42" customHeight="1">
+        <x:v>Melee ability. Cast. Range 1.50. Physical damage (weapon damage + Strength x100%). Radius 1.50 around caster; click caster to confirm. Affects: enemies. Melee weapon required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="57" customHeight="1">
       <x:c r="A11" s="22" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -929,16 +929,16 @@
         <x:v>Warrior</x:v>
       </x:c>
       <x:c r="C11" s="22" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D11" s="23" t="str">
-        <x:v>Multi Attack</x:v>
+        <x:v>Taunt</x:v>
       </x:c>
       <x:c r="E11" s="23" t="str">
-        <x:v>Melee ability. Melee. Range 1.41. Physical damage (2 hits × (weapon damage + Strength x50%)). 2 separate hits on the same target. Affects: enemies. Melee weapon required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="72" customHeight="1">
+        <x:v>Melee ability. Cast. Range 1.50. Taunted: Attack the caster if possible; otherwise pursue them for 1 turn. Negative status. Radius 1.50 around caster; click caster to confirm. Affects: enemies. No weapon required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="18" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -946,16 +946,16 @@
         <x:v>Warrior</x:v>
       </x:c>
       <x:c r="C12" s="18" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>Counter</x:v>
+        <x:v>Multi Attack</x:v>
       </x:c>
       <x:c r="E12" s="19" t="str">
-        <x:v>Melee ability. Cast. Range 0.00. Counter for 1 turn. After each complete damaging attack, retaliate once with your basic attack if the attacker is in range. Retaliation costs no action or opportunity reaction. Requires being able to attack; excludes terrain, damage over time, and other counters. Expires at next turn start. Positive status. Affects: self. No weapon required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="57" customHeight="1">
+        <x:v>Melee ability. Melee. Range 1.41. Physical damage (2 hits × (weapon damage + Strength x50%)). 2 separate hits on the same target. Affects: enemies. Melee weapon required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="72" customHeight="1">
       <x:c r="A13" s="22" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -963,16 +963,16 @@
         <x:v>Warrior</x:v>
       </x:c>
       <x:c r="C13" s="22" t="n">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D13" s="23" t="str">
-        <x:v>Swipe</x:v>
+        <x:v>Counter</x:v>
       </x:c>
       <x:c r="E13" s="23" t="str">
-        <x:v>Melee ability. Melee. Range 1.00. Physical damage (weapon damage + Strength x100%). Click an orthogonally adjacent cell; hit a 3-cell row across that direction. Affects: enemies. Can aim at a cell. Area: line in front, 3-cell span. Melee weapon required.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="72" customHeight="1">
+        <x:v>Melee ability. Cast. Range 0.00. Counter for 1 turn. After each complete damaging attack, retaliate once with your basic attack if the attacker is in range. Retaliation costs no action or opportunity reaction. Requires being able to attack; excludes terrain, damage over time, and other counters. Expires at next turn start. Positive status. Affects: self. No weapon required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="57" customHeight="1">
       <x:c r="A14" s="18" t="n">
         <x:v>9</x:v>
       </x:c>
@@ -980,12 +980,29 @@
         <x:v>Warrior</x:v>
       </x:c>
       <x:c r="C14" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D14" s="19" t="str">
+        <x:v>Swipe</x:v>
+      </x:c>
+      <x:c r="E14" s="19" t="str">
+        <x:v>Melee ability. Melee. Range 1.00. Physical damage (weapon damage + Strength x100%). Click an orthogonally adjacent cell; hit a 3-cell row across that direction. Affects: enemies. Can aim at a cell. Area: line in front, 3-cell span. Melee weapon required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="22" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B15" s="23" t="str">
+        <x:v>Warrior</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D14" s="19" t="str">
+      <x:c r="D15" s="23" t="str">
         <x:v>Ram</x:v>
       </x:c>
-      <x:c r="E14" s="19" t="str">
+      <x:c r="E15" s="23" t="str">
         <x:v>Melee ability. Melee. Range 1.00. Physical damage (Strength x100%), Push up to 2 tiles away; walls and board edges deal 1 collision damage; hitting a unit stops the push and deals 1 to both (armor applies). No chain push, terrain entry effects, or opportunity attacks. Affects: enemies. No weapon required.</x:v>
       </x:c>
     </x:row>
@@ -995,7 +1012,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c00eeaddc924b30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fc3614299014f96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1192,7 +1209,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R092dd6e20e594019"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra002b15ebf594dde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>